<commit_message>
Fase 185: Tipificación de WhatsApp de ORLANT por fecha de cierre (v1.74.0)
- HistChat: el día de cada chat sale de DATE_CLOSE (Wolkvox arma el archivo
  por fecha de cierre). Los chats abiertos el último día del mes anterior ya
  no se van a ese mes ni borran ese día al reemplazar el rango.
- Tarjeta "Total WhatsApp"; resumen por causa de las filas omitidas; DATE
  "dd/mm/aaaa hh:mm" ya se lee.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/server/plantillas/PLANTILLA_TIPIFICACION_WHATSAPP.xlsx
+++ b/server/plantillas/PLANTILLA_TIPIFICACION_WHATSAPP.xlsx
@@ -560,7 +560,7 @@
         <v>De dónde sale</v>
       </c>
       <c r="B2" t="str">
-        <v>Wolkvox: CDR de WhatsApp, export "HistChat&lt;fecha&gt;" — [ruta pendiente de confirmar con Edwin]. Se sube tal cual (no hay que renombrar la hoja); el sistema nunca lee nombres, correos, teléfonos ni el texto de las conversaciones. Un SKILL_ID que no esté en la tabla de skills se ignora y la vista previa dice cuántos.</v>
+        <v>Wolkvox: CDR de WhatsApp, export "HistChat&lt;fecha&gt;" — [ruta pendiente de confirmar con Edwin]. Se sube tal cual (no hay que renombrar la hoja); el sistema nunca lee nombres, correos, teléfonos ni el texto de las conversaciones. Un SKILL_ID que no esté en la tabla de skills se guarda como "Skill &lt;número&gt;" y la vista previa dice cuántos. El día de cada chat sale de DATE_CLOSE (fecha de cierre).</v>
       </c>
     </row>
     <row r="3">
@@ -662,7 +662,7 @@
         <v>Sí</v>
       </c>
       <c r="C12" t="str">
-        <v>Fecha y hora de la conversación.</v>
+        <v>Fecha y hora de apertura del chat. Solo se usa si la fila no trae DATE_CLOSE.</v>
       </c>
       <c r="D12" t="str">
         <v>2026-09-01 08:15:00</v>
@@ -679,7 +679,7 @@
         <v>No</v>
       </c>
       <c r="C13" t="str">
-        <v>Viene en el export de Wolkvox; el sistema no la usa.</v>
+        <v>Fecha y hora de cierre: define el día y el mes del chat (Wolkvox arma el archivo por fecha de cierre).</v>
       </c>
       <c r="D13" t="str">
         <v>2026-09-01 08:30:00</v>

</xml_diff>